<commit_message>
Import Pi Desktop/Recurve production tree.
Capture the running shop Pi (605002B-2) Recurve folder into git so GitHub
matches what is deployed, including kiosk boot scripts and Wi-Fi transfer tweaks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Data_Files/Test.xlsx
+++ b/Data_Files/Test.xlsx
@@ -46,8 +46,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,79 +416,119 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr"/>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Prox. OD (inch)</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Dist. OD (inch)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Dist. Cone Length (mm)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Body Length (mm)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ΦA1 (mm)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ΦA2 (mm)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ΦA3 (mm)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Prox. Cone Length (mm)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Body Length (mm)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>ΦA1 (mm)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ΦA2 (mm)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ΦA3 (mm)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Dist. Cone Length (mm)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Dist.OD (inch)</t>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Prox.OD (inch)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="1" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>0.043</v>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="n">
         <v>0.042</v>
       </c>
-      <c r="C2" t="n">
-        <v>41.09</v>
-      </c>
-      <c r="D2" t="n">
-        <v>37.28</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="H2" t="n">
-        <v>14.67</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.042</v>
+      <c r="C3" s="1" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>32.67</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>